<commit_message>
LectureTable, needs conversion in pandas
</commit_message>
<xml_diff>
--- a/LectureTable.xlsx
+++ b/LectureTable.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Desktop\Embedded Intelligence\D7065E\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB97609F-4DF5-4548-9C74-A525ED62B365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62A434C7-7E60-4F32-9770-4B23E7AEF463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3990" yWindow="2790" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,23 +26,64 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>classroom</t>
-  </si>
-  <si>
-    <t>schedule</t>
-  </si>
-  <si>
-    <t>a109</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="13">
+  <si>
+    <t>A109</t>
+  </si>
+  <si>
+    <t>Lektion</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Starttid</t>
+  </si>
+  <si>
+    <t>Sluttid</t>
+  </si>
+  <si>
+    <t>Dag</t>
+  </si>
+  <si>
+    <t>Klassrum</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>Slut</t>
+  </si>
+  <si>
+    <t>Måndag</t>
+  </si>
+  <si>
+    <t>Nej</t>
+  </si>
+  <si>
+    <t>A110</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="hh:mm;@"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -69,8 +111,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -351,19 +413,250 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="3" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6">
+        <v>0.34375</v>
+      </c>
+      <c r="C2" s="6">
+        <v>0.40625</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.48958333333333331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25719DD1-ECCE-4EF2-8834-D6E7ABB26DBA}">
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="D2" s="6">
+        <v>0.34375</v>
+      </c>
+      <c r="E2" s="6">
+        <v>0.40625</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0.34375</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0.40625</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="E8" s="6">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>